<commit_message>
Added the Sam Core ISA in its current state in the spreadsheet
</commit_message>
<xml_diff>
--- a/sam_isa.xlsx
+++ b/sam_isa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t xml:space="preserve">SAM CPU Core ISA</t>
   </si>
@@ -50,6 +50,84 @@
   </si>
   <si>
     <t xml:space="preserve">&lt; Low Nibble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUB #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIV #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUL #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AND #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORA #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOR #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XNR #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUB $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIV $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUL $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AND $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORA $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOR $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XNR $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDA #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDA $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STA $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JZ $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HLT</t>
   </si>
 </sst>
 </file>
@@ -64,6 +142,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -147,36 +226,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -368,7 +451,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
+      <c r="B1" s="2"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -390,14 +473,14 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="2"/>
+      <c r="E2" s="3"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -416,444 +499,496 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="P3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="R3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="S3" s="4" t="s">
         <v>9</v>
       </c>
       <c r="T3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="8"/>
       <c r="T4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="8"/>
       <c r="T5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="7"/>
+      <c r="C6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="8"/>
       <c r="T6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="8"/>
       <c r="T7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="8"/>
       <c r="T8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="7"/>
+      <c r="C9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="S9" s="8"/>
       <c r="T9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="8"/>
       <c r="T10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="8"/>
       <c r="T11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="8"/>
       <c r="T12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
+      <c r="S13" s="8"/>
       <c r="T13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="6"/>
-      <c r="S14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="7"/>
+      <c r="S14" s="8"/>
       <c r="T14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="7"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="8"/>
       <c r="T15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="6"/>
-      <c r="R16" s="6"/>
-      <c r="S16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="8"/>
       <c r="T16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="8"/>
       <c r="T17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="6"/>
-      <c r="Q18" s="6"/>
-      <c r="R18" s="6"/>
-      <c r="S18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="8"/>
       <c r="T18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="6"/>
-      <c r="P19" s="6"/>
-      <c r="Q19" s="6"/>
-      <c r="R19" s="6"/>
-      <c r="S19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S19" s="8"/>
       <c r="T19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Updated Sam core ISA
</commit_message>
<xml_diff>
--- a/sam_isa.xlsx
+++ b/sam_isa.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ISA" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="ISA Breakdown" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="118">
   <si>
     <t xml:space="preserve">SAM CPU Core ISA</t>
   </si>
@@ -118,6 +119,9 @@
     <t xml:space="preserve">JZ $</t>
   </si>
   <si>
+    <t xml:space="preserve">MOV</t>
+  </si>
+  <si>
     <t xml:space="preserve">INC</t>
   </si>
   <si>
@@ -128,6 +132,249 @@
   </si>
   <si>
     <t xml:space="preserve">HLT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arithmetic Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mnemonic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opcode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDA#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Accumulator from Immediate (2 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No operation this cycle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDA$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Accumulator from Absolute Address (3 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0xFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halt CPU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUB#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtract immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STA$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store Accumulator to Absolute Address (3 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increment Accumulator by 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUB$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtract absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unconditional Jump to Address (3 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decrement Accumulator by 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIV#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divide Immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JZ$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jump to Address if Zero Flag is 1 (3 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x5F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Output Accumulator to IO (3 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIV$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divide Absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy value from one register to another (3 bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUL#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiply Immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUL$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiply Absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AND#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise AND immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AND$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise AND absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORA#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise OR immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORA$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise OR absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOR#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise XOR immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOR$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise XOR absolute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XNR#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise XNOR immediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XNR$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise XNOR absolute</t>
   </si>
 </sst>
 </file>
@@ -160,7 +407,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -191,13 +438,32 @@
         <bgColor rgb="FFEC9BA4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFDBB6"/>
+        <bgColor rgb="FFFFD8CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD8CE"/>
+        <bgColor rgb="FFFFDBB6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -226,7 +492,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -263,6 +529,18 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -292,7 +570,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFD8CE"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -313,11 +591,11 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFEC9BA4"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFB66C"/>
+      <rgbColor rgb="FFFFDBB6"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFFB66C"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
@@ -702,7 +980,9 @@
       <c r="D8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="7"/>
+      <c r="E8" s="7" t="s">
+        <v>32</v>
+      </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
@@ -725,10 +1005,10 @@
         <v>5</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -744,7 +1024,7 @@
       <c r="P9" s="7"/>
       <c r="Q9" s="7"/>
       <c r="R9" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S9" s="8"/>
       <c r="T9" s="1"/>
@@ -986,7 +1266,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="7"/>
       <c r="R19" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S19" s="8"/>
       <c r="T19" s="1"/>
@@ -1032,4 +1312,648 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:T19"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="H1" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="O1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="H2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="O2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="H3" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="O3" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="P3" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="H4" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="O4" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q4" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
+      <c r="T4" s="11"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="H5" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="O5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="H6" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="O6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="P6" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q6" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="R6" s="11"/>
+      <c r="S6" s="11"/>
+      <c r="T6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="H7" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="O7" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="P7" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q7" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="R7" s="11"/>
+      <c r="S7" s="11"/>
+      <c r="T7" s="11"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="H8" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
+      <c r="S8" s="11"/>
+      <c r="T8" s="11"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11"/>
+      <c r="T9" s="11"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11"/>
+      <c r="T10" s="11"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="11"/>
+      <c r="T12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="11"/>
+      <c r="S13" s="11"/>
+      <c r="T13" s="11"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="11"/>
+      <c r="S14" s="11"/>
+      <c r="T14" s="11"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
+      <c r="T15" s="11"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="11"/>
+      <c r="S16" s="11"/>
+      <c r="T16" s="11"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="11"/>
+      <c r="T17" s="11"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="11"/>
+      <c r="S18" s="11"/>
+      <c r="T18" s="11"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="11"/>
+      <c r="R19" s="11"/>
+      <c r="S19" s="11"/>
+      <c r="T19" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="57">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="O1:T1"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="Q3:T3"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="Q4:T4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="Q5:T5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="Q6:T6"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="Q7:T7"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="Q8:T8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="Q9:T9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="Q10:T10"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="Q11:T11"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="J12:M12"/>
+    <mergeCell ref="Q12:T12"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="Q14:T14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="J15:M15"/>
+    <mergeCell ref="Q15:T15"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="J16:M16"/>
+    <mergeCell ref="Q16:T16"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="Q17:T17"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="J18:M18"/>
+    <mergeCell ref="Q18:T18"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="J19:M19"/>
+    <mergeCell ref="Q19:T19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>